<commit_message>
Updating data dictionary 4/7/2026
</commit_message>
<xml_diff>
--- a/Data Dictionaries (Upload Here)/SDE/SDE_Data_Dictionary.xlsx
+++ b/Data Dictionaries (Upload Here)/SDE/SDE_Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctgovexec.sharepoint.com/sites/SDEEdSight/Shared Documents/General/Data Requests/P20WIN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="8_{F85219D9-2FDE-4689-BA90-4A31AB0F38EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB4A007F-7D62-495D-B51D-D863E4D3A181}"/>
+  <xr:revisionPtr revIDLastSave="110" documentId="8_{F85219D9-2FDE-4689-BA90-4A31AB0F38EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5754B0E-6BE8-45F3-A60C-1EB3E3917E10}"/>
   <bookViews>
-    <workbookView xWindow="-51720" yWindow="-3255" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core" sheetId="17" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="338">
   <si>
     <t>Agency</t>
   </si>
@@ -363,9 +363,6 @@
   </si>
   <si>
     <t>End date for the period of enrollment</t>
-  </si>
-  <si>
-    <t>Type of college that the student attended: 4 = 4-year or higher institution; 2 = 2-year institution; L = less than 2-year institution</t>
   </si>
   <si>
     <t>EnrollmentStatus</t>
@@ -1073,6 +1070,9 @@
   </si>
   <si>
     <t>Specific to the facility attended at the time of reporting, the total number of instructional days a student has been enrolled for the current school year. Only reported for Collection = June.</t>
+  </si>
+  <si>
+    <t>Type of college that the student graduated from: 4 = 4-year or higher institution; 2 = 2-year institution; L = less than 2-year institution</t>
   </si>
 </sst>
 </file>
@@ -1460,13 +1460,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B96AA09A-2052-45AD-BBA4-E66D63D93DA6}">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G152"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="34.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="26" style="1" customWidth="1"/>
-    <col min="4" max="4" width="124" style="1" customWidth="1"/>
+    <col min="4" max="4" width="43.28515625" style="1" customWidth="1"/>
     <col min="5" max="5" width="171.28515625" style="1" customWidth="1"/>
     <col min="6" max="6" width="19.140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="33.28515625" style="1" customWidth="1"/>
@@ -1483,16 +1483,16 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F1" t="s">
         <v>124</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>167</v>
-      </c>
-      <c r="F1" t="s">
-        <v>125</v>
-      </c>
-      <c r="G1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1813,10 +1813,10 @@
         <v>19</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>328</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>329</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>43</v>
@@ -1977,7 +1977,7 @@
         <v>75</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>21</v>
@@ -2000,7 +2000,7 @@
         <v>76</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>21</v>
@@ -2023,7 +2023,7 @@
         <v>77</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>45</v>
@@ -2201,7 +2201,7 @@
         <v>4</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>20</v>
@@ -2224,16 +2224,16 @@
         <v>4</v>
       </c>
       <c r="C34" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="D34" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="E34" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>331</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>332</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>73</v>
@@ -2523,7 +2523,7 @@
         <v>4</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>20</v>
@@ -2546,10 +2546,10 @@
         <v>4</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>107</v>
@@ -2569,10 +2569,10 @@
         <v>4</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>108</v>
@@ -2592,13 +2592,13 @@
         <v>4</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D50" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E50" s="4" t="s">
         <v>324</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>325</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>103</v>
@@ -2615,13 +2615,13 @@
         <v>4</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D51" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E51" s="5" t="s">
         <v>110</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>111</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>69</v>
@@ -2638,7 +2638,7 @@
         <v>4</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>20</v>
@@ -2661,13 +2661,13 @@
         <v>4</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>109</v>
+        <v>337</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>103</v>
@@ -2684,12 +2684,12 @@
         <v>4</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E54" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>111</v>
       </c>
       <c r="F54" s="1" t="s">
@@ -2707,16 +2707,16 @@
         <v>4</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>112</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>106</v>
@@ -2730,7 +2730,7 @@
         <v>4</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>326</v>
@@ -2739,7 +2739,7 @@
         <v>113</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>106</v>
@@ -2753,19 +2753,19 @@
         <v>4</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="D57" s="3" t="s">
-        <v>327</v>
+        <v>114</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>114</v>
+        <v>22</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>106</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
@@ -2776,13 +2776,13 @@
         <v>4</v>
       </c>
       <c r="C58" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E58" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>21</v>
@@ -2799,16 +2799,16 @@
         <v>4</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>21</v>
+        <v>117</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>23</v>
@@ -2822,16 +2822,16 @@
         <v>4</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D60" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>23</v>
@@ -2845,16 +2845,16 @@
         <v>4</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>23</v>
@@ -2868,183 +2868,181 @@
         <v>4</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>122</v>
+        <v>335</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>123</v>
+        <v>334</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>336</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="A63" t="s">
+        <v>174</v>
+      </c>
+      <c r="B63" t="s">
+        <v>125</v>
+      </c>
+      <c r="C63" t="s">
+        <v>170</v>
+      </c>
+      <c r="D63" t="s">
+        <v>175</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="F63" t="s">
+        <v>177</v>
+      </c>
+      <c r="G63"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B64" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C64" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D64" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F64" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G64"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B65" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C65" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D65" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E65" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="F65" t="s">
         <v>180</v>
-      </c>
-      <c r="F65" t="s">
-        <v>181</v>
       </c>
       <c r="G65"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B66" t="s">
+        <v>125</v>
+      </c>
+      <c r="C66" t="s">
+        <v>170</v>
+      </c>
+      <c r="D66" t="s">
         <v>126</v>
-      </c>
-      <c r="C66" t="s">
-        <v>171</v>
-      </c>
-      <c r="D66" t="s">
-        <v>182</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>183</v>
       </c>
       <c r="F66" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="G66"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B67" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C67" t="s">
+        <v>170</v>
+      </c>
+      <c r="D67" t="s">
         <v>171</v>
       </c>
-      <c r="D67" t="s">
-        <v>127</v>
-      </c>
       <c r="E67" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F67" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="G67"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B68" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C68" t="s">
-        <v>171</v>
+        <v>125</v>
       </c>
       <c r="D68" t="s">
-        <v>172</v>
-      </c>
-      <c r="E68" s="6" t="s">
         <v>186</v>
       </c>
+      <c r="E68" s="6"/>
       <c r="F68" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="G68"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B69" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C69" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D69" t="s">
         <v>187</v>
       </c>
-      <c r="E69" s="6"/>
+      <c r="E69" s="6" t="s">
+        <v>169</v>
+      </c>
       <c r="F69" t="s">
-        <v>185</v>
+        <v>80</v>
       </c>
       <c r="G69"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B70" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C70" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D70" t="s">
         <v>188</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F70" t="s">
         <v>80</v>
@@ -3053,19 +3051,19 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B71" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C71" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D71" t="s">
         <v>189</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="F71" t="s">
         <v>80</v>
@@ -3074,20 +3072,18 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B72" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C72" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D72" t="s">
-        <v>190</v>
-      </c>
-      <c r="E72" s="6" t="s">
         <v>191</v>
       </c>
+      <c r="E72" s="6"/>
       <c r="F72" t="s">
         <v>80</v>
       </c>
@@ -3095,95 +3091,97 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B73" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C73" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D73" t="s">
         <v>192</v>
       </c>
-      <c r="E73" s="6"/>
+      <c r="E73" s="6" t="s">
+        <v>193</v>
+      </c>
       <c r="F73" t="s">
-        <v>80</v>
+        <v>194</v>
       </c>
       <c r="G73"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B74" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C74" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D74" t="s">
-        <v>193</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>194</v>
+        <v>127</v>
+      </c>
+      <c r="E74" t="s">
+        <v>195</v>
       </c>
       <c r="F74" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G74"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B75" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C75" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D75" t="s">
-        <v>128</v>
+        <v>197</v>
       </c>
       <c r="E75" t="s">
+        <v>198</v>
+      </c>
+      <c r="F75" t="s">
         <v>196</v>
-      </c>
-      <c r="F75" t="s">
-        <v>197</v>
       </c>
       <c r="G75"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B76" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C76" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D76" t="s">
-        <v>198</v>
+        <v>128</v>
       </c>
       <c r="E76" t="s">
         <v>199</v>
       </c>
       <c r="F76" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G76"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B77" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C77" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D77" t="s">
         <v>129</v>
@@ -3192,61 +3190,61 @@
         <v>200</v>
       </c>
       <c r="F77" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G77"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B78" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C78" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D78" t="s">
         <v>130</v>
       </c>
-      <c r="E78" t="s">
+      <c r="E78" s="6" t="s">
         <v>201</v>
       </c>
       <c r="F78" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G78"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B79" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C79" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D79" t="s">
         <v>131</v>
       </c>
-      <c r="E79" s="6" t="s">
+      <c r="E79" t="s">
         <v>202</v>
       </c>
       <c r="F79" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G79"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B80" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C80" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D80" t="s">
         <v>132</v>
@@ -3255,82 +3253,82 @@
         <v>203</v>
       </c>
       <c r="F80" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="G80"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B81" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C81" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D81" t="s">
         <v>133</v>
       </c>
       <c r="E81" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F81" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="G81"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B82" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C82" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D82" t="s">
         <v>134</v>
       </c>
-      <c r="E82" t="s">
+      <c r="E82" s="6" t="s">
         <v>206</v>
       </c>
       <c r="F82" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G82"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B83" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C83" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D83" t="s">
         <v>135</v>
       </c>
-      <c r="E83" s="6" t="s">
+      <c r="E83" t="s">
         <v>207</v>
       </c>
       <c r="F83" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G83"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B84" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C84" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D84" t="s">
         <v>136</v>
@@ -3339,208 +3337,208 @@
         <v>208</v>
       </c>
       <c r="F84" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="G84"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B85" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C85" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D85" t="s">
-        <v>137</v>
+        <v>210</v>
       </c>
       <c r="E85" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F85" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="G85"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B86" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C86" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D86" t="s">
-        <v>211</v>
-      </c>
-      <c r="E86" t="s">
         <v>212</v>
       </c>
+      <c r="E86" s="6" t="s">
+        <v>213</v>
+      </c>
       <c r="F86" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G86"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B87" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C87" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D87" t="s">
-        <v>213</v>
-      </c>
-      <c r="E87" s="6" t="s">
         <v>214</v>
       </c>
+      <c r="E87" t="s">
+        <v>215</v>
+      </c>
       <c r="F87" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G87"/>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B88" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C88" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D88" t="s">
-        <v>215</v>
+        <v>137</v>
       </c>
       <c r="E88" t="s">
         <v>216</v>
       </c>
       <c r="F88" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G88"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B89" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C89" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D89" t="s">
-        <v>138</v>
-      </c>
-      <c r="E89" t="s">
         <v>217</v>
       </c>
+      <c r="E89" s="7" t="s">
+        <v>218</v>
+      </c>
       <c r="F89" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G89"/>
     </row>
-    <row r="90" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B90" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C90" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D90" t="s">
-        <v>218</v>
-      </c>
-      <c r="E90" s="7" t="s">
         <v>219</v>
       </c>
+      <c r="E90" t="s">
+        <v>220</v>
+      </c>
       <c r="F90" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G90"/>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B91" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C91" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D91" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E91" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F91" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G91"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B92" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C92" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D92" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E92" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F92" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G92"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B93" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C93" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D93" t="s">
-        <v>224</v>
+        <v>138</v>
       </c>
       <c r="E93" t="s">
         <v>225</v>
       </c>
       <c r="F93" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G93"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B94" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C94" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D94" t="s">
         <v>139</v>
@@ -3549,19 +3547,19 @@
         <v>226</v>
       </c>
       <c r="F94" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G94"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B95" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C95" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D95" t="s">
         <v>140</v>
@@ -3570,19 +3568,19 @@
         <v>227</v>
       </c>
       <c r="F95" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G95"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B96" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C96" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D96" t="s">
         <v>141</v>
@@ -3591,19 +3589,19 @@
         <v>228</v>
       </c>
       <c r="F96" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G96"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B97" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C97" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D97" t="s">
         <v>142</v>
@@ -3612,19 +3610,19 @@
         <v>229</v>
       </c>
       <c r="F97" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G97"/>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B98" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C98" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D98" t="s">
         <v>143</v>
@@ -3633,19 +3631,19 @@
         <v>230</v>
       </c>
       <c r="F98" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="G98"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B99" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C99" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D99" t="s">
         <v>144</v>
@@ -3654,775 +3652,775 @@
         <v>231</v>
       </c>
       <c r="F99" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G99"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B100" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C100" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D100" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="E100" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F100" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="G100"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B101" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C101" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D101" t="s">
-        <v>233</v>
-      </c>
-      <c r="E101" t="s">
         <v>234</v>
       </c>
+      <c r="E101" s="6" t="s">
+        <v>235</v>
+      </c>
       <c r="F101" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G101"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B102" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C102" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D102" t="s">
-        <v>235</v>
-      </c>
-      <c r="E102" s="6" t="s">
         <v>236</v>
       </c>
+      <c r="E102" t="s">
+        <v>237</v>
+      </c>
       <c r="F102" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G102"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B103" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C103" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D103" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E103" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F103" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G103"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B104" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C104" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D104" t="s">
-        <v>239</v>
-      </c>
-      <c r="E104" t="s">
         <v>240</v>
       </c>
+      <c r="E104" s="6" t="s">
+        <v>241</v>
+      </c>
       <c r="F104" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G104"/>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B105" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C105" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D105" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F105" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G105"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B106" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C106" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D106" t="s">
-        <v>243</v>
-      </c>
-      <c r="E106" s="6" t="s">
         <v>244</v>
       </c>
+      <c r="E106" t="s">
+        <v>245</v>
+      </c>
       <c r="F106" t="s">
-        <v>197</v>
+        <v>246</v>
       </c>
       <c r="G106"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B107" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C107" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D107" t="s">
-        <v>245</v>
-      </c>
-      <c r="E107" t="s">
-        <v>246</v>
+        <v>145</v>
+      </c>
+      <c r="E107" s="6" t="s">
+        <v>247</v>
       </c>
       <c r="F107" t="s">
-        <v>247</v>
+        <v>209</v>
       </c>
       <c r="G107"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B108" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C108" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D108" t="s">
-        <v>146</v>
+        <v>248</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F108" t="s">
-        <v>210</v>
+        <v>184</v>
       </c>
       <c r="G108"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B109" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C109" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D109" t="s">
-        <v>249</v>
-      </c>
-      <c r="E109" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="E109" t="s">
         <v>250</v>
       </c>
       <c r="F109" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="G109"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B110" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C110" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D110" t="s">
-        <v>147</v>
+        <v>251</v>
       </c>
       <c r="E110" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F110" t="s">
-        <v>197</v>
+        <v>253</v>
       </c>
       <c r="G110"/>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B111" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C111" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D111" t="s">
-        <v>252</v>
+        <v>147</v>
       </c>
       <c r="E111" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F111" t="s">
-        <v>254</v>
+        <v>184</v>
       </c>
       <c r="G111"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B112" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C112" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D112" t="s">
-        <v>148</v>
+        <v>255</v>
       </c>
       <c r="E112" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F112" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="G112"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B113" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C113" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D113" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E113" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F113" t="s">
-        <v>210</v>
+        <v>259</v>
       </c>
       <c r="G113"/>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B114" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C114" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D114" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E114" t="s">
-        <v>259</v>
+        <v>319</v>
       </c>
       <c r="F114" t="s">
-        <v>260</v>
-      </c>
-      <c r="G114"/>
+        <v>261</v>
+      </c>
+      <c r="G114" s="8"/>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B115" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C115" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D115" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E115" t="s">
-        <v>320</v>
+        <v>263</v>
       </c>
       <c r="F115" t="s">
-        <v>262</v>
-      </c>
-      <c r="G115" s="8"/>
+        <v>209</v>
+      </c>
+      <c r="G115"/>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B116" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C116" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D116" t="s">
-        <v>263</v>
-      </c>
-      <c r="E116" t="s">
         <v>264</v>
       </c>
+      <c r="E116" s="6" t="s">
+        <v>265</v>
+      </c>
       <c r="F116" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G116"/>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B117" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C117" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D117" t="s">
-        <v>265</v>
+        <v>148</v>
       </c>
       <c r="E117" s="6" t="s">
         <v>266</v>
       </c>
       <c r="F117" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="G117"/>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B118" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C118" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D118" t="s">
-        <v>149</v>
-      </c>
-      <c r="E118" s="6" t="s">
         <v>267</v>
       </c>
+      <c r="E118" t="s">
+        <v>268</v>
+      </c>
       <c r="F118" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G118"/>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B119" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C119" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D119" t="s">
-        <v>268</v>
-      </c>
-      <c r="E119" t="s">
         <v>269</v>
       </c>
+      <c r="E119" s="6" t="s">
+        <v>270</v>
+      </c>
       <c r="F119" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G119"/>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B120" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C120" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D120" t="s">
-        <v>270</v>
-      </c>
-      <c r="E120" s="6" t="s">
         <v>271</v>
       </c>
+      <c r="E120" t="s">
+        <v>272</v>
+      </c>
       <c r="F120" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="G120"/>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B121" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C121" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D121" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E121" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F121" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="G121"/>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B122" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C122" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D122" t="s">
-        <v>274</v>
-      </c>
-      <c r="E122" t="s">
         <v>275</v>
       </c>
+      <c r="E122" s="6" t="s">
+        <v>276</v>
+      </c>
       <c r="F122" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G122"/>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B123" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C123" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D123" t="s">
-        <v>276</v>
+        <v>149</v>
       </c>
       <c r="E123" s="6" t="s">
         <v>277</v>
       </c>
       <c r="F123" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G123"/>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B124" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C124" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D124" t="s">
-        <v>150</v>
+        <v>278</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F124" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G124"/>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B125" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C125" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D125" t="s">
-        <v>279</v>
-      </c>
-      <c r="E125" s="6" t="s">
         <v>280</v>
       </c>
+      <c r="E125" t="s">
+        <v>281</v>
+      </c>
       <c r="F125" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G125"/>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B126" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C126" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D126" t="s">
-        <v>281</v>
-      </c>
-      <c r="E126" t="s">
         <v>282</v>
       </c>
+      <c r="E126" s="6" t="s">
+        <v>283</v>
+      </c>
       <c r="F126" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G126"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B127" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C127" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D127" t="s">
-        <v>283</v>
-      </c>
-      <c r="E127" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="E127" t="s">
         <v>284</v>
       </c>
       <c r="F127" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G127"/>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B128" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C128" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D128" t="s">
-        <v>151</v>
+        <v>285</v>
       </c>
       <c r="E128" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F128" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G128"/>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B129" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C129" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D129" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E129" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F129" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="G129"/>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B130" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C130" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D130" t="s">
-        <v>288</v>
+        <v>151</v>
       </c>
       <c r="E130" t="s">
         <v>289</v>
       </c>
       <c r="F130" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="G130"/>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B131" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C131" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D131" t="s">
-        <v>152</v>
+        <v>290</v>
       </c>
       <c r="E131" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F131" t="s">
-        <v>197</v>
+        <v>292</v>
       </c>
       <c r="G131"/>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B132" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C132" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D132" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E132" t="s">
+        <v>294</v>
+      </c>
+      <c r="F132" t="s">
         <v>292</v>
-      </c>
-      <c r="F132" t="s">
-        <v>293</v>
       </c>
       <c r="G132"/>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B133" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C133" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D133" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E133" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F133" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G133"/>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B134" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C134" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D134" t="s">
-        <v>296</v>
-      </c>
-      <c r="E134" t="s">
         <v>297</v>
       </c>
+      <c r="E134" s="6" t="s">
+        <v>298</v>
+      </c>
       <c r="F134" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G134"/>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B135" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C135" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D135" t="s">
-        <v>298</v>
-      </c>
-      <c r="E135" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="E135" t="s">
         <v>299</v>
       </c>
       <c r="F135" t="s">
-        <v>293</v>
+        <v>196</v>
       </c>
       <c r="G135"/>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B136" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C136" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D136" t="s">
         <v>153</v>
@@ -4431,19 +4429,19 @@
         <v>300</v>
       </c>
       <c r="F136" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="G136"/>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B137" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C137" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D137" t="s">
         <v>154</v>
@@ -4452,19 +4450,19 @@
         <v>301</v>
       </c>
       <c r="F137" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="G137"/>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B138" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C138" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D138" t="s">
         <v>155</v>
@@ -4473,61 +4471,61 @@
         <v>302</v>
       </c>
       <c r="F138" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="G138"/>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B139" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C139" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D139" t="s">
         <v>156</v>
       </c>
       <c r="E139" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="F139" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="G139"/>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B140" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C140" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D140" t="s">
         <v>157</v>
       </c>
       <c r="E140" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F140" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="G140"/>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B141" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C141" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D141" t="s">
         <v>158</v>
@@ -4536,19 +4534,19 @@
         <v>304</v>
       </c>
       <c r="F141" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G141"/>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B142" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C142" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D142" t="s">
         <v>159</v>
@@ -4557,61 +4555,61 @@
         <v>305</v>
       </c>
       <c r="F142" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G142"/>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B143" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C143" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D143" t="s">
         <v>160</v>
       </c>
-      <c r="E143" t="s">
+      <c r="E143" s="6" t="s">
         <v>306</v>
       </c>
       <c r="F143" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G143"/>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B144" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C144" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D144" t="s">
         <v>161</v>
       </c>
-      <c r="E144" s="6" t="s">
+      <c r="E144" t="s">
         <v>307</v>
       </c>
       <c r="F144" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G144"/>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B145" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C145" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D145" t="s">
         <v>162</v>
@@ -4620,177 +4618,156 @@
         <v>308</v>
       </c>
       <c r="F145" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G145"/>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B146" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C146" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D146" t="s">
-        <v>163</v>
+        <v>309</v>
       </c>
       <c r="E146" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F146" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G146"/>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B147" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C147" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D147" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E147" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F147" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G147"/>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B148" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C148" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D148" t="s">
-        <v>312</v>
+        <v>163</v>
       </c>
       <c r="E148" t="s">
         <v>313</v>
       </c>
       <c r="F148" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G148"/>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B149" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C149" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D149" t="s">
-        <v>164</v>
-      </c>
-      <c r="E149" t="s">
         <v>314</v>
       </c>
+      <c r="E149" s="6" t="s">
+        <v>315</v>
+      </c>
       <c r="F149" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="G149"/>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B150" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C150" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D150" t="s">
+        <v>316</v>
+      </c>
+      <c r="E150" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="E150" s="6" t="s">
-        <v>316</v>
-      </c>
       <c r="F150" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G150"/>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B151" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C151" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D151" t="s">
+        <v>165</v>
+      </c>
+      <c r="E151" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E151" s="6" t="s">
-        <v>316</v>
-      </c>
       <c r="F151" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G151"/>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B152" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C152" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D152" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>318</v>
       </c>
       <c r="F152" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="G152"/>
-    </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
-        <v>175</v>
-      </c>
-      <c r="B153" t="s">
-        <v>126</v>
-      </c>
-      <c r="C153" t="s">
-        <v>126</v>
-      </c>
-      <c r="D153" t="s">
-        <v>165</v>
-      </c>
-      <c r="E153" s="6" t="s">
-        <v>319</v>
-      </c>
-      <c r="F153" t="s">
-        <v>185</v>
-      </c>
-      <c r="G153"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4798,6 +4775,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="7fe1ab5a-1809-4ce3-b80e-370d008aa218" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4cf662d2-5748-4aa1-b153-5e852749b621">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A6925AA43B38B14C9EB09FF1C1C42642" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bb16190c67cfe802431256201a21c7c5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4cf662d2-5748-4aa1-b153-5e852749b621" xmlns:ns3="7fe1ab5a-1809-4ce3-b80e-370d008aa218" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="596d067d5548c93e8fb0f26023627946" ns2:_="" ns3:_="">
     <xsd:import namespace="4cf662d2-5748-4aa1-b153-5e852749b621"/>
@@ -5032,17 +5020,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="7fe1ab5a-1809-4ce3-b80e-370d008aa218" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4cf662d2-5748-4aa1-b153-5e852749b621">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -5053,6 +5030,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A3D2406E-606D-4AA1-8036-D5637B960319}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="7fe1ab5a-1809-4ce3-b80e-370d008aa218"/>
+    <ds:schemaRef ds:uri="4cf662d2-5748-4aa1-b153-5e852749b621"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{337ACD63-2331-4622-A069-203CF9E93252}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5071,17 +5059,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A3D2406E-606D-4AA1-8036-D5637B960319}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="7fe1ab5a-1809-4ce3-b80e-370d008aa218"/>
-    <ds:schemaRef ds:uri="4cf662d2-5748-4aa1-b153-5e852749b621"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FA153C3-0472-4559-920C-F4452307722A}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update 4/22/2026, correct Agency name
</commit_message>
<xml_diff>
--- a/Data Dictionaries (Upload Here)/SDE/SDE_Data_Dictionary.xlsx
+++ b/Data Dictionaries (Upload Here)/SDE/SDE_Data_Dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctgovexec.sharepoint.com/sites/SDEEdSight/Shared Documents/General/Data Requests/P20WIN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="8_{F85219D9-2FDE-4689-BA90-4A31AB0F38EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5754B0E-6BE8-45F3-A60C-1EB3E3917E10}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="8_{F85219D9-2FDE-4689-BA90-4A31AB0F38EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1076F06D-6690-47FE-A6C6-1CCF7C902F27}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="337">
   <si>
     <t>Agency</t>
   </si>
@@ -558,9 +558,6 @@
   </si>
   <si>
     <t>College - NSC - Graduation</t>
-  </si>
-  <si>
-    <t>State Department of Education</t>
   </si>
   <si>
     <t>Student ID / Unique Individual Identifier (PIRL Element 100)</t>
@@ -1461,18 +1458,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B96AA09A-2052-45AD-BBA4-E66D63D93DA6}">
   <dimension ref="A1:G152"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="34.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="60.36328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="34.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="26" style="1" customWidth="1"/>
-    <col min="4" max="4" width="43.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="171.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="33.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="117.7265625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="171.26953125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="33.26953125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1495,7 +1492,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1515,7 +1512,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1535,7 +1532,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1555,7 +1552,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1575,7 +1572,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1595,7 +1592,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1618,7 +1615,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1641,7 +1638,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -1664,7 +1661,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1687,7 +1684,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
@@ -1710,7 +1707,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>3</v>
       </c>
@@ -1733,7 +1730,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>3</v>
       </c>
@@ -1756,7 +1753,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>3</v>
       </c>
@@ -1779,7 +1776,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
@@ -1802,7 +1799,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1813,10 +1810,10 @@
         <v>19</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>327</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>328</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>43</v>
@@ -1825,7 +1822,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
@@ -1848,7 +1845,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>3</v>
       </c>
@@ -1871,7 +1868,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>3</v>
       </c>
@@ -1894,7 +1891,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>3</v>
       </c>
@@ -1917,7 +1914,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>3</v>
       </c>
@@ -1940,7 +1937,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
@@ -1963,7 +1960,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>3</v>
       </c>
@@ -1977,7 +1974,7 @@
         <v>75</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>21</v>
@@ -1986,7 +1983,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>3</v>
       </c>
@@ -2000,7 +1997,7 @@
         <v>76</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>21</v>
@@ -2009,7 +2006,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>3</v>
       </c>
@@ -2023,7 +2020,7 @@
         <v>77</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>45</v>
@@ -2032,7 +2029,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>3</v>
       </c>
@@ -2055,7 +2052,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>3</v>
       </c>
@@ -2078,7 +2075,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>3</v>
       </c>
@@ -2101,7 +2098,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>3</v>
       </c>
@@ -2124,7 +2121,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>3</v>
       </c>
@@ -2147,7 +2144,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>3</v>
       </c>
@@ -2170,7 +2167,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>3</v>
       </c>
@@ -2193,7 +2190,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>3</v>
       </c>
@@ -2201,7 +2198,7 @@
         <v>4</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>20</v>
@@ -2216,7 +2213,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>3</v>
       </c>
@@ -2224,22 +2221,22 @@
         <v>4</v>
       </c>
       <c r="C34" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="D34" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="E34" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>330</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>331</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>3</v>
       </c>
@@ -2262,7 +2259,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>3</v>
       </c>
@@ -2285,7 +2282,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>3</v>
       </c>
@@ -2308,7 +2305,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>3</v>
       </c>
@@ -2331,7 +2328,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>3</v>
       </c>
@@ -2354,7 +2351,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>3</v>
       </c>
@@ -2377,7 +2374,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>3</v>
       </c>
@@ -2400,7 +2397,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>3</v>
       </c>
@@ -2423,7 +2420,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>3</v>
       </c>
@@ -2446,7 +2443,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>3</v>
       </c>
@@ -2469,7 +2466,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>3</v>
       </c>
@@ -2492,7 +2489,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>3</v>
       </c>
@@ -2515,7 +2512,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>3</v>
       </c>
@@ -2538,7 +2535,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>3</v>
       </c>
@@ -2549,7 +2546,7 @@
         <v>172</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>107</v>
@@ -2561,7 +2558,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>3</v>
       </c>
@@ -2572,7 +2569,7 @@
         <v>172</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>108</v>
@@ -2584,7 +2581,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>3</v>
       </c>
@@ -2595,10 +2592,10 @@
         <v>172</v>
       </c>
       <c r="D50" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="E50" s="4" t="s">
         <v>323</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>324</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>103</v>
@@ -2607,7 +2604,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>3</v>
       </c>
@@ -2630,7 +2627,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>3</v>
       </c>
@@ -2653,7 +2650,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>3</v>
       </c>
@@ -2664,10 +2661,10 @@
         <v>173</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>103</v>
@@ -2676,7 +2673,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>3</v>
       </c>
@@ -2687,7 +2684,7 @@
         <v>173</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>111</v>
@@ -2699,7 +2696,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>3</v>
       </c>
@@ -2710,7 +2707,7 @@
         <v>173</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>112</v>
@@ -2722,7 +2719,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>3</v>
       </c>
@@ -2733,7 +2730,7 @@
         <v>173</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>113</v>
@@ -2745,7 +2742,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>3</v>
       </c>
@@ -2768,7 +2765,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>3</v>
       </c>
@@ -2791,7 +2788,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>3</v>
       </c>
@@ -2814,7 +2811,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>3</v>
       </c>
@@ -2837,7 +2834,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>3</v>
       </c>
@@ -2860,7 +2857,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>3</v>
       </c>
@@ -2871,10 +2868,10 @@
         <v>114</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>117</v>
@@ -2883,9 +2880,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>174</v>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B63" t="s">
         <v>125</v>
@@ -2894,19 +2891,19 @@
         <v>170</v>
       </c>
       <c r="D63" t="s">
+        <v>174</v>
+      </c>
+      <c r="E63" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="E63" s="6" t="s">
+      <c r="F63" t="s">
         <v>176</v>
       </c>
-      <c r="F63" t="s">
-        <v>177</v>
-      </c>
       <c r="G63"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>174</v>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B64" t="s">
         <v>125</v>
@@ -2915,19 +2912,19 @@
         <v>170</v>
       </c>
       <c r="D64" t="s">
+        <v>177</v>
+      </c>
+      <c r="E64" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="E64" s="6" t="s">
+      <c r="F64" t="s">
         <v>179</v>
       </c>
-      <c r="F64" t="s">
-        <v>180</v>
-      </c>
       <c r="G64"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>174</v>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B65" t="s">
         <v>125</v>
@@ -2936,19 +2933,19 @@
         <v>170</v>
       </c>
       <c r="D65" t="s">
+        <v>180</v>
+      </c>
+      <c r="E65" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="E65" s="6" t="s">
-        <v>182</v>
-      </c>
       <c r="F65" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G65"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>174</v>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B66" t="s">
         <v>125</v>
@@ -2960,16 +2957,16 @@
         <v>126</v>
       </c>
       <c r="E66" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="F66" t="s">
         <v>183</v>
       </c>
-      <c r="F66" t="s">
-        <v>184</v>
-      </c>
       <c r="G66"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>174</v>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B67" t="s">
         <v>125</v>
@@ -2981,35 +2978,35 @@
         <v>171</v>
       </c>
       <c r="E67" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="F67" t="s">
+        <v>179</v>
+      </c>
+      <c r="G67"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B68" t="s">
+        <v>125</v>
+      </c>
+      <c r="C68" t="s">
+        <v>125</v>
+      </c>
+      <c r="D68" t="s">
         <v>185</v>
-      </c>
-      <c r="F67" t="s">
-        <v>180</v>
-      </c>
-      <c r="G67"/>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>174</v>
-      </c>
-      <c r="B68" t="s">
-        <v>125</v>
-      </c>
-      <c r="C68" t="s">
-        <v>125</v>
-      </c>
-      <c r="D68" t="s">
-        <v>186</v>
       </c>
       <c r="E68" s="6"/>
       <c r="F68" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G68"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>174</v>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B69" t="s">
         <v>125</v>
@@ -3018,7 +3015,7 @@
         <v>125</v>
       </c>
       <c r="D69" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>169</v>
@@ -3028,9 +3025,9 @@
       </c>
       <c r="G69"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>174</v>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B70" t="s">
         <v>125</v>
@@ -3039,7 +3036,7 @@
         <v>125</v>
       </c>
       <c r="D70" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>168</v>
@@ -3049,9 +3046,9 @@
       </c>
       <c r="G70"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>174</v>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B71" t="s">
         <v>125</v>
@@ -3060,19 +3057,19 @@
         <v>125</v>
       </c>
       <c r="D71" t="s">
+        <v>188</v>
+      </c>
+      <c r="E71" s="6" t="s">
         <v>189</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>190</v>
       </c>
       <c r="F71" t="s">
         <v>80</v>
       </c>
       <c r="G71"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>174</v>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B72" t="s">
         <v>125</v>
@@ -3081,7 +3078,7 @@
         <v>125</v>
       </c>
       <c r="D72" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E72" s="6"/>
       <c r="F72" t="s">
@@ -3089,9 +3086,9 @@
       </c>
       <c r="G72"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>174</v>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B73" t="s">
         <v>125</v>
@@ -3100,19 +3097,19 @@
         <v>125</v>
       </c>
       <c r="D73" t="s">
+        <v>191</v>
+      </c>
+      <c r="E73" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="E73" s="6" t="s">
+      <c r="F73" t="s">
         <v>193</v>
       </c>
-      <c r="F73" t="s">
-        <v>194</v>
-      </c>
       <c r="G73"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>174</v>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A74" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B74" t="s">
         <v>125</v>
@@ -3124,37 +3121,37 @@
         <v>127</v>
       </c>
       <c r="E74" t="s">
+        <v>194</v>
+      </c>
+      <c r="F74" t="s">
         <v>195</v>
       </c>
-      <c r="F74" t="s">
+      <c r="G74"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A75" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B75" t="s">
+        <v>125</v>
+      </c>
+      <c r="C75" t="s">
+        <v>125</v>
+      </c>
+      <c r="D75" t="s">
         <v>196</v>
       </c>
-      <c r="G74"/>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>174</v>
-      </c>
-      <c r="B75" t="s">
-        <v>125</v>
-      </c>
-      <c r="C75" t="s">
-        <v>125</v>
-      </c>
-      <c r="D75" t="s">
+      <c r="E75" t="s">
         <v>197</v>
       </c>
-      <c r="E75" t="s">
-        <v>198</v>
-      </c>
       <c r="F75" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G75"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>174</v>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A76" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B76" t="s">
         <v>125</v>
@@ -3166,16 +3163,16 @@
         <v>128</v>
       </c>
       <c r="E76" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F76" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G76"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>174</v>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A77" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B77" t="s">
         <v>125</v>
@@ -3187,16 +3184,16 @@
         <v>129</v>
       </c>
       <c r="E77" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F77" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G77"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>174</v>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A78" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B78" t="s">
         <v>125</v>
@@ -3208,16 +3205,16 @@
         <v>130</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F78" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G78"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>174</v>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A79" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B79" t="s">
         <v>125</v>
@@ -3229,16 +3226,16 @@
         <v>131</v>
       </c>
       <c r="E79" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F79" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G79"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>174</v>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A80" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B80" t="s">
         <v>125</v>
@@ -3250,16 +3247,16 @@
         <v>132</v>
       </c>
       <c r="E80" t="s">
+        <v>202</v>
+      </c>
+      <c r="F80" t="s">
         <v>203</v>
       </c>
-      <c r="F80" t="s">
-        <v>204</v>
-      </c>
       <c r="G80"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>174</v>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A81" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B81" t="s">
         <v>125</v>
@@ -3271,16 +3268,16 @@
         <v>133</v>
       </c>
       <c r="E81" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F81" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G81"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>174</v>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A82" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B82" t="s">
         <v>125</v>
@@ -3292,16 +3289,16 @@
         <v>134</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F82" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G82"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>174</v>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A83" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B83" t="s">
         <v>125</v>
@@ -3313,16 +3310,16 @@
         <v>135</v>
       </c>
       <c r="E83" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F83" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G83"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>174</v>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A84" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B84" t="s">
         <v>125</v>
@@ -3334,79 +3331,79 @@
         <v>136</v>
       </c>
       <c r="E84" t="s">
+        <v>207</v>
+      </c>
+      <c r="F84" t="s">
         <v>208</v>
       </c>
-      <c r="F84" t="s">
+      <c r="G84"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A85" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B85" t="s">
+        <v>125</v>
+      </c>
+      <c r="C85" t="s">
+        <v>125</v>
+      </c>
+      <c r="D85" t="s">
         <v>209</v>
       </c>
-      <c r="G84"/>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>174</v>
-      </c>
-      <c r="B85" t="s">
-        <v>125</v>
-      </c>
-      <c r="C85" t="s">
-        <v>125</v>
-      </c>
-      <c r="D85" t="s">
+      <c r="E85" t="s">
         <v>210</v>
       </c>
-      <c r="E85" t="s">
+      <c r="F85" t="s">
+        <v>195</v>
+      </c>
+      <c r="G85"/>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A86" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B86" t="s">
+        <v>125</v>
+      </c>
+      <c r="C86" t="s">
+        <v>125</v>
+      </c>
+      <c r="D86" t="s">
         <v>211</v>
       </c>
-      <c r="F85" t="s">
-        <v>196</v>
-      </c>
-      <c r="G85"/>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>174</v>
-      </c>
-      <c r="B86" t="s">
-        <v>125</v>
-      </c>
-      <c r="C86" t="s">
-        <v>125</v>
-      </c>
-      <c r="D86" t="s">
+      <c r="E86" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="E86" s="6" t="s">
+      <c r="F86" t="s">
+        <v>195</v>
+      </c>
+      <c r="G86"/>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A87" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B87" t="s">
+        <v>125</v>
+      </c>
+      <c r="C87" t="s">
+        <v>125</v>
+      </c>
+      <c r="D87" t="s">
         <v>213</v>
       </c>
-      <c r="F86" t="s">
-        <v>196</v>
-      </c>
-      <c r="G86"/>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>174</v>
-      </c>
-      <c r="B87" t="s">
-        <v>125</v>
-      </c>
-      <c r="C87" t="s">
-        <v>125</v>
-      </c>
-      <c r="D87" t="s">
+      <c r="E87" t="s">
         <v>214</v>
       </c>
-      <c r="E87" t="s">
-        <v>215</v>
-      </c>
       <c r="F87" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G87"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>174</v>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A88" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B88" t="s">
         <v>125</v>
@@ -3418,100 +3415,100 @@
         <v>137</v>
       </c>
       <c r="E88" t="s">
+        <v>215</v>
+      </c>
+      <c r="F88" t="s">
+        <v>195</v>
+      </c>
+      <c r="G88"/>
+    </row>
+    <row r="89" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A89" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B89" t="s">
+        <v>125</v>
+      </c>
+      <c r="C89" t="s">
+        <v>125</v>
+      </c>
+      <c r="D89" t="s">
         <v>216</v>
       </c>
-      <c r="F88" t="s">
-        <v>196</v>
-      </c>
-      <c r="G88"/>
-    </row>
-    <row r="89" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>174</v>
-      </c>
-      <c r="B89" t="s">
-        <v>125</v>
-      </c>
-      <c r="C89" t="s">
-        <v>125</v>
-      </c>
-      <c r="D89" t="s">
+      <c r="E89" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="E89" s="7" t="s">
+      <c r="F89" t="s">
+        <v>195</v>
+      </c>
+      <c r="G89"/>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A90" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B90" t="s">
+        <v>125</v>
+      </c>
+      <c r="C90" t="s">
+        <v>125</v>
+      </c>
+      <c r="D90" t="s">
         <v>218</v>
       </c>
-      <c r="F89" t="s">
-        <v>196</v>
-      </c>
-      <c r="G89"/>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>174</v>
-      </c>
-      <c r="B90" t="s">
-        <v>125</v>
-      </c>
-      <c r="C90" t="s">
-        <v>125</v>
-      </c>
-      <c r="D90" t="s">
+      <c r="E90" t="s">
         <v>219</v>
       </c>
-      <c r="E90" t="s">
+      <c r="F90" t="s">
+        <v>195</v>
+      </c>
+      <c r="G90"/>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A91" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B91" t="s">
+        <v>125</v>
+      </c>
+      <c r="C91" t="s">
+        <v>125</v>
+      </c>
+      <c r="D91" t="s">
         <v>220</v>
       </c>
-      <c r="F90" t="s">
-        <v>196</v>
-      </c>
-      <c r="G90"/>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>174</v>
-      </c>
-      <c r="B91" t="s">
-        <v>125</v>
-      </c>
-      <c r="C91" t="s">
-        <v>125</v>
-      </c>
-      <c r="D91" t="s">
+      <c r="E91" t="s">
         <v>221</v>
       </c>
-      <c r="E91" t="s">
+      <c r="F91" t="s">
+        <v>195</v>
+      </c>
+      <c r="G91"/>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A92" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B92" t="s">
+        <v>125</v>
+      </c>
+      <c r="C92" t="s">
+        <v>125</v>
+      </c>
+      <c r="D92" t="s">
         <v>222</v>
       </c>
-      <c r="F91" t="s">
-        <v>196</v>
-      </c>
-      <c r="G91"/>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>174</v>
-      </c>
-      <c r="B92" t="s">
-        <v>125</v>
-      </c>
-      <c r="C92" t="s">
-        <v>125</v>
-      </c>
-      <c r="D92" t="s">
+      <c r="E92" t="s">
         <v>223</v>
       </c>
-      <c r="E92" t="s">
-        <v>224</v>
-      </c>
       <c r="F92" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G92"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>174</v>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A93" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B93" t="s">
         <v>125</v>
@@ -3523,16 +3520,16 @@
         <v>138</v>
       </c>
       <c r="E93" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F93" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G93"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>174</v>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A94" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B94" t="s">
         <v>125</v>
@@ -3544,16 +3541,16 @@
         <v>139</v>
       </c>
       <c r="E94" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F94" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G94"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>174</v>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A95" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B95" t="s">
         <v>125</v>
@@ -3565,16 +3562,16 @@
         <v>140</v>
       </c>
       <c r="E95" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F95" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G95"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>174</v>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A96" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B96" t="s">
         <v>125</v>
@@ -3586,16 +3583,16 @@
         <v>141</v>
       </c>
       <c r="E96" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F96" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G96"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>174</v>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A97" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B97" t="s">
         <v>125</v>
@@ -3607,16 +3604,16 @@
         <v>142</v>
       </c>
       <c r="E97" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F97" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G97"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>174</v>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A98" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B98" t="s">
         <v>125</v>
@@ -3628,16 +3625,16 @@
         <v>143</v>
       </c>
       <c r="E98" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F98" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G98"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>174</v>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A99" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B99" t="s">
         <v>125</v>
@@ -3649,163 +3646,163 @@
         <v>144</v>
       </c>
       <c r="E99" t="s">
+        <v>230</v>
+      </c>
+      <c r="F99" t="s">
+        <v>183</v>
+      </c>
+      <c r="G99"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A100" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B100" t="s">
+        <v>125</v>
+      </c>
+      <c r="C100" t="s">
+        <v>125</v>
+      </c>
+      <c r="D100" t="s">
         <v>231</v>
       </c>
-      <c r="F99" t="s">
-        <v>184</v>
-      </c>
-      <c r="G99"/>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>174</v>
-      </c>
-      <c r="B100" t="s">
-        <v>125</v>
-      </c>
-      <c r="C100" t="s">
-        <v>125</v>
-      </c>
-      <c r="D100" t="s">
+      <c r="E100" t="s">
         <v>232</v>
       </c>
-      <c r="E100" t="s">
+      <c r="F100" t="s">
+        <v>195</v>
+      </c>
+      <c r="G100"/>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A101" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B101" t="s">
+        <v>125</v>
+      </c>
+      <c r="C101" t="s">
+        <v>125</v>
+      </c>
+      <c r="D101" t="s">
         <v>233</v>
       </c>
-      <c r="F100" t="s">
-        <v>196</v>
-      </c>
-      <c r="G100"/>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>174</v>
-      </c>
-      <c r="B101" t="s">
-        <v>125</v>
-      </c>
-      <c r="C101" t="s">
-        <v>125</v>
-      </c>
-      <c r="D101" t="s">
+      <c r="E101" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="E101" s="6" t="s">
+      <c r="F101" t="s">
+        <v>195</v>
+      </c>
+      <c r="G101"/>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A102" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B102" t="s">
+        <v>125</v>
+      </c>
+      <c r="C102" t="s">
+        <v>125</v>
+      </c>
+      <c r="D102" t="s">
         <v>235</v>
       </c>
-      <c r="F101" t="s">
-        <v>196</v>
-      </c>
-      <c r="G101"/>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>174</v>
-      </c>
-      <c r="B102" t="s">
-        <v>125</v>
-      </c>
-      <c r="C102" t="s">
-        <v>125</v>
-      </c>
-      <c r="D102" t="s">
+      <c r="E102" t="s">
         <v>236</v>
       </c>
-      <c r="E102" t="s">
+      <c r="F102" t="s">
+        <v>195</v>
+      </c>
+      <c r="G102"/>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A103" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B103" t="s">
+        <v>125</v>
+      </c>
+      <c r="C103" t="s">
+        <v>125</v>
+      </c>
+      <c r="D103" t="s">
         <v>237</v>
       </c>
-      <c r="F102" t="s">
-        <v>196</v>
-      </c>
-      <c r="G102"/>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>174</v>
-      </c>
-      <c r="B103" t="s">
-        <v>125</v>
-      </c>
-      <c r="C103" t="s">
-        <v>125</v>
-      </c>
-      <c r="D103" t="s">
+      <c r="E103" t="s">
         <v>238</v>
       </c>
-      <c r="E103" t="s">
+      <c r="F103" t="s">
+        <v>195</v>
+      </c>
+      <c r="G103"/>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A104" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B104" t="s">
+        <v>125</v>
+      </c>
+      <c r="C104" t="s">
+        <v>125</v>
+      </c>
+      <c r="D104" t="s">
         <v>239</v>
       </c>
-      <c r="F103" t="s">
-        <v>196</v>
-      </c>
-      <c r="G103"/>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>174</v>
-      </c>
-      <c r="B104" t="s">
-        <v>125</v>
-      </c>
-      <c r="C104" t="s">
-        <v>125</v>
-      </c>
-      <c r="D104" t="s">
+      <c r="E104" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="E104" s="6" t="s">
+      <c r="F104" t="s">
+        <v>195</v>
+      </c>
+      <c r="G104"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A105" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B105" t="s">
+        <v>125</v>
+      </c>
+      <c r="C105" t="s">
+        <v>125</v>
+      </c>
+      <c r="D105" t="s">
         <v>241</v>
       </c>
-      <c r="F104" t="s">
-        <v>196</v>
-      </c>
-      <c r="G104"/>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>174</v>
-      </c>
-      <c r="B105" t="s">
-        <v>125</v>
-      </c>
-      <c r="C105" t="s">
-        <v>125</v>
-      </c>
-      <c r="D105" t="s">
+      <c r="E105" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="E105" s="6" t="s">
+      <c r="F105" t="s">
+        <v>195</v>
+      </c>
+      <c r="G105"/>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A106" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B106" t="s">
+        <v>125</v>
+      </c>
+      <c r="C106" t="s">
+        <v>125</v>
+      </c>
+      <c r="D106" t="s">
         <v>243</v>
       </c>
-      <c r="F105" t="s">
-        <v>196</v>
-      </c>
-      <c r="G105"/>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>174</v>
-      </c>
-      <c r="B106" t="s">
-        <v>125</v>
-      </c>
-      <c r="C106" t="s">
-        <v>125</v>
-      </c>
-      <c r="D106" t="s">
+      <c r="E106" t="s">
         <v>244</v>
       </c>
-      <c r="E106" t="s">
+      <c r="F106" t="s">
         <v>245</v>
       </c>
-      <c r="F106" t="s">
-        <v>246</v>
-      </c>
       <c r="G106"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>174</v>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A107" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B107" t="s">
         <v>125</v>
@@ -3817,37 +3814,37 @@
         <v>145</v>
       </c>
       <c r="E107" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="F107" t="s">
+        <v>208</v>
+      </c>
+      <c r="G107"/>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A108" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B108" t="s">
+        <v>125</v>
+      </c>
+      <c r="C108" t="s">
+        <v>125</v>
+      </c>
+      <c r="D108" t="s">
         <v>247</v>
       </c>
-      <c r="F107" t="s">
-        <v>209</v>
-      </c>
-      <c r="G107"/>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>174</v>
-      </c>
-      <c r="B108" t="s">
-        <v>125</v>
-      </c>
-      <c r="C108" t="s">
-        <v>125</v>
-      </c>
-      <c r="D108" t="s">
+      <c r="E108" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="E108" s="6" t="s">
-        <v>249</v>
-      </c>
       <c r="F108" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G108"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>174</v>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A109" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B109" t="s">
         <v>125</v>
@@ -3859,37 +3856,37 @@
         <v>146</v>
       </c>
       <c r="E109" t="s">
+        <v>249</v>
+      </c>
+      <c r="F109" t="s">
+        <v>195</v>
+      </c>
+      <c r="G109"/>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A110" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B110" t="s">
+        <v>125</v>
+      </c>
+      <c r="C110" t="s">
+        <v>125</v>
+      </c>
+      <c r="D110" t="s">
         <v>250</v>
       </c>
-      <c r="F109" t="s">
-        <v>196</v>
-      </c>
-      <c r="G109"/>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>174</v>
-      </c>
-      <c r="B110" t="s">
-        <v>125</v>
-      </c>
-      <c r="C110" t="s">
-        <v>125</v>
-      </c>
-      <c r="D110" t="s">
+      <c r="E110" t="s">
         <v>251</v>
       </c>
-      <c r="E110" t="s">
+      <c r="F110" t="s">
         <v>252</v>
       </c>
-      <c r="F110" t="s">
-        <v>253</v>
-      </c>
       <c r="G110"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>174</v>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A111" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B111" t="s">
         <v>125</v>
@@ -3901,121 +3898,121 @@
         <v>147</v>
       </c>
       <c r="E111" t="s">
+        <v>253</v>
+      </c>
+      <c r="F111" t="s">
+        <v>183</v>
+      </c>
+      <c r="G111"/>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A112" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B112" t="s">
+        <v>125</v>
+      </c>
+      <c r="C112" t="s">
+        <v>125</v>
+      </c>
+      <c r="D112" t="s">
         <v>254</v>
       </c>
-      <c r="F111" t="s">
-        <v>184</v>
-      </c>
-      <c r="G111"/>
-    </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>174</v>
-      </c>
-      <c r="B112" t="s">
-        <v>125</v>
-      </c>
-      <c r="C112" t="s">
-        <v>125</v>
-      </c>
-      <c r="D112" t="s">
+      <c r="E112" t="s">
         <v>255</v>
       </c>
-      <c r="E112" t="s">
+      <c r="F112" t="s">
+        <v>208</v>
+      </c>
+      <c r="G112"/>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A113" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B113" t="s">
+        <v>125</v>
+      </c>
+      <c r="C113" t="s">
+        <v>125</v>
+      </c>
+      <c r="D113" t="s">
         <v>256</v>
       </c>
-      <c r="F112" t="s">
-        <v>209</v>
-      </c>
-      <c r="G112"/>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>174</v>
-      </c>
-      <c r="B113" t="s">
-        <v>125</v>
-      </c>
-      <c r="C113" t="s">
-        <v>125</v>
-      </c>
-      <c r="D113" t="s">
+      <c r="E113" t="s">
         <v>257</v>
       </c>
-      <c r="E113" t="s">
+      <c r="F113" t="s">
         <v>258</v>
       </c>
-      <c r="F113" t="s">
+      <c r="G113"/>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A114" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B114" t="s">
+        <v>125</v>
+      </c>
+      <c r="C114" t="s">
+        <v>125</v>
+      </c>
+      <c r="D114" t="s">
         <v>259</v>
       </c>
-      <c r="G113"/>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>174</v>
-      </c>
-      <c r="B114" t="s">
-        <v>125</v>
-      </c>
-      <c r="C114" t="s">
-        <v>125</v>
-      </c>
-      <c r="D114" t="s">
+      <c r="E114" t="s">
+        <v>318</v>
+      </c>
+      <c r="F114" t="s">
         <v>260</v>
       </c>
-      <c r="E114" t="s">
-        <v>319</v>
-      </c>
-      <c r="F114" t="s">
+      <c r="G114" s="8"/>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A115" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B115" t="s">
+        <v>125</v>
+      </c>
+      <c r="C115" t="s">
+        <v>125</v>
+      </c>
+      <c r="D115" t="s">
         <v>261</v>
       </c>
-      <c r="G114" s="8"/>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>174</v>
-      </c>
-      <c r="B115" t="s">
-        <v>125</v>
-      </c>
-      <c r="C115" t="s">
-        <v>125</v>
-      </c>
-      <c r="D115" t="s">
+      <c r="E115" t="s">
         <v>262</v>
       </c>
-      <c r="E115" t="s">
+      <c r="F115" t="s">
+        <v>208</v>
+      </c>
+      <c r="G115"/>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A116" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B116" t="s">
+        <v>125</v>
+      </c>
+      <c r="C116" t="s">
+        <v>125</v>
+      </c>
+      <c r="D116" t="s">
         <v>263</v>
       </c>
-      <c r="F115" t="s">
-        <v>209</v>
-      </c>
-      <c r="G115"/>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>174</v>
-      </c>
-      <c r="B116" t="s">
-        <v>125</v>
-      </c>
-      <c r="C116" t="s">
-        <v>125</v>
-      </c>
-      <c r="D116" t="s">
+      <c r="E116" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="E116" s="6" t="s">
-        <v>265</v>
-      </c>
       <c r="F116" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G116"/>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>174</v>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A117" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B117" t="s">
         <v>125</v>
@@ -4027,121 +4024,121 @@
         <v>148</v>
       </c>
       <c r="E117" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="F117" t="s">
+        <v>195</v>
+      </c>
+      <c r="G117"/>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A118" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B118" t="s">
+        <v>125</v>
+      </c>
+      <c r="C118" t="s">
+        <v>125</v>
+      </c>
+      <c r="D118" t="s">
         <v>266</v>
       </c>
-      <c r="F117" t="s">
-        <v>196</v>
-      </c>
-      <c r="G117"/>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>174</v>
-      </c>
-      <c r="B118" t="s">
-        <v>125</v>
-      </c>
-      <c r="C118" t="s">
-        <v>125</v>
-      </c>
-      <c r="D118" t="s">
+      <c r="E118" t="s">
         <v>267</v>
       </c>
-      <c r="E118" t="s">
+      <c r="F118" t="s">
+        <v>195</v>
+      </c>
+      <c r="G118"/>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A119" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B119" t="s">
+        <v>125</v>
+      </c>
+      <c r="C119" t="s">
+        <v>125</v>
+      </c>
+      <c r="D119" t="s">
         <v>268</v>
       </c>
-      <c r="F118" t="s">
-        <v>196</v>
-      </c>
-      <c r="G118"/>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>174</v>
-      </c>
-      <c r="B119" t="s">
-        <v>125</v>
-      </c>
-      <c r="C119" t="s">
-        <v>125</v>
-      </c>
-      <c r="D119" t="s">
+      <c r="E119" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="E119" s="6" t="s">
+      <c r="F119" t="s">
+        <v>195</v>
+      </c>
+      <c r="G119"/>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A120" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B120" t="s">
+        <v>125</v>
+      </c>
+      <c r="C120" t="s">
+        <v>125</v>
+      </c>
+      <c r="D120" t="s">
         <v>270</v>
       </c>
-      <c r="F119" t="s">
-        <v>196</v>
-      </c>
-      <c r="G119"/>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>174</v>
-      </c>
-      <c r="B120" t="s">
-        <v>125</v>
-      </c>
-      <c r="C120" t="s">
-        <v>125</v>
-      </c>
-      <c r="D120" t="s">
+      <c r="E120" t="s">
         <v>271</v>
       </c>
-      <c r="E120" t="s">
+      <c r="F120" t="s">
+        <v>183</v>
+      </c>
+      <c r="G120"/>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A121" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B121" t="s">
+        <v>125</v>
+      </c>
+      <c r="C121" t="s">
+        <v>125</v>
+      </c>
+      <c r="D121" t="s">
         <v>272</v>
       </c>
-      <c r="F120" t="s">
-        <v>184</v>
-      </c>
-      <c r="G120"/>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>174</v>
-      </c>
-      <c r="B121" t="s">
-        <v>125</v>
-      </c>
-      <c r="C121" t="s">
-        <v>125</v>
-      </c>
-      <c r="D121" t="s">
+      <c r="E121" t="s">
         <v>273</v>
       </c>
-      <c r="E121" t="s">
+      <c r="F121" t="s">
+        <v>195</v>
+      </c>
+      <c r="G121"/>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A122" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B122" t="s">
+        <v>125</v>
+      </c>
+      <c r="C122" t="s">
+        <v>125</v>
+      </c>
+      <c r="D122" t="s">
         <v>274</v>
       </c>
-      <c r="F121" t="s">
-        <v>196</v>
-      </c>
-      <c r="G121"/>
-    </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>174</v>
-      </c>
-      <c r="B122" t="s">
-        <v>125</v>
-      </c>
-      <c r="C122" t="s">
-        <v>125</v>
-      </c>
-      <c r="D122" t="s">
+      <c r="E122" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="E122" s="6" t="s">
-        <v>276</v>
-      </c>
       <c r="F122" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G122"/>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>174</v>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A123" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B123" t="s">
         <v>125</v>
@@ -4153,79 +4150,79 @@
         <v>149</v>
       </c>
       <c r="E123" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="F123" t="s">
+        <v>195</v>
+      </c>
+      <c r="G123"/>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A124" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B124" t="s">
+        <v>125</v>
+      </c>
+      <c r="C124" t="s">
+        <v>125</v>
+      </c>
+      <c r="D124" t="s">
         <v>277</v>
       </c>
-      <c r="F123" t="s">
-        <v>196</v>
-      </c>
-      <c r="G123"/>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>174</v>
-      </c>
-      <c r="B124" t="s">
-        <v>125</v>
-      </c>
-      <c r="C124" t="s">
-        <v>125</v>
-      </c>
-      <c r="D124" t="s">
+      <c r="E124" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="E124" s="6" t="s">
+      <c r="F124" t="s">
+        <v>195</v>
+      </c>
+      <c r="G124"/>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A125" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B125" t="s">
+        <v>125</v>
+      </c>
+      <c r="C125" t="s">
+        <v>125</v>
+      </c>
+      <c r="D125" t="s">
         <v>279</v>
       </c>
-      <c r="F124" t="s">
-        <v>196</v>
-      </c>
-      <c r="G124"/>
-    </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>174</v>
-      </c>
-      <c r="B125" t="s">
-        <v>125</v>
-      </c>
-      <c r="C125" t="s">
-        <v>125</v>
-      </c>
-      <c r="D125" t="s">
+      <c r="E125" t="s">
         <v>280</v>
       </c>
-      <c r="E125" t="s">
+      <c r="F125" t="s">
+        <v>195</v>
+      </c>
+      <c r="G125"/>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A126" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B126" t="s">
+        <v>125</v>
+      </c>
+      <c r="C126" t="s">
+        <v>125</v>
+      </c>
+      <c r="D126" t="s">
         <v>281</v>
       </c>
-      <c r="F125" t="s">
-        <v>196</v>
-      </c>
-      <c r="G125"/>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>174</v>
-      </c>
-      <c r="B126" t="s">
-        <v>125</v>
-      </c>
-      <c r="C126" t="s">
-        <v>125</v>
-      </c>
-      <c r="D126" t="s">
+      <c r="E126" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="E126" s="6" t="s">
-        <v>283</v>
-      </c>
       <c r="F126" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G126"/>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>174</v>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A127" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B127" t="s">
         <v>125</v>
@@ -4237,58 +4234,58 @@
         <v>150</v>
       </c>
       <c r="E127" t="s">
+        <v>283</v>
+      </c>
+      <c r="F127" t="s">
+        <v>195</v>
+      </c>
+      <c r="G127"/>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A128" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B128" t="s">
+        <v>125</v>
+      </c>
+      <c r="C128" t="s">
+        <v>125</v>
+      </c>
+      <c r="D128" t="s">
         <v>284</v>
       </c>
-      <c r="F127" t="s">
-        <v>196</v>
-      </c>
-      <c r="G127"/>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>174</v>
-      </c>
-      <c r="B128" t="s">
-        <v>125</v>
-      </c>
-      <c r="C128" t="s">
-        <v>125</v>
-      </c>
-      <c r="D128" t="s">
+      <c r="E128" t="s">
         <v>285</v>
       </c>
-      <c r="E128" t="s">
+      <c r="F128" t="s">
+        <v>195</v>
+      </c>
+      <c r="G128"/>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A129" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B129" t="s">
+        <v>125</v>
+      </c>
+      <c r="C129" t="s">
+        <v>125</v>
+      </c>
+      <c r="D129" t="s">
         <v>286</v>
       </c>
-      <c r="F128" t="s">
-        <v>196</v>
-      </c>
-      <c r="G128"/>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
-        <v>174</v>
-      </c>
-      <c r="B129" t="s">
-        <v>125</v>
-      </c>
-      <c r="C129" t="s">
-        <v>125</v>
-      </c>
-      <c r="D129" t="s">
+      <c r="E129" t="s">
         <v>287</v>
       </c>
-      <c r="E129" t="s">
-        <v>288</v>
-      </c>
       <c r="F129" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G129"/>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
-        <v>174</v>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A130" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B130" t="s">
         <v>125</v>
@@ -4300,100 +4297,100 @@
         <v>151</v>
       </c>
       <c r="E130" t="s">
+        <v>288</v>
+      </c>
+      <c r="F130" t="s">
+        <v>195</v>
+      </c>
+      <c r="G130"/>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A131" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B131" t="s">
+        <v>125</v>
+      </c>
+      <c r="C131" t="s">
+        <v>125</v>
+      </c>
+      <c r="D131" t="s">
         <v>289</v>
       </c>
-      <c r="F130" t="s">
-        <v>196</v>
-      </c>
-      <c r="G130"/>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
-        <v>174</v>
-      </c>
-      <c r="B131" t="s">
-        <v>125</v>
-      </c>
-      <c r="C131" t="s">
-        <v>125</v>
-      </c>
-      <c r="D131" t="s">
+      <c r="E131" t="s">
         <v>290</v>
       </c>
-      <c r="E131" t="s">
+      <c r="F131" t="s">
         <v>291</v>
       </c>
-      <c r="F131" t="s">
+      <c r="G131"/>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A132" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B132" t="s">
+        <v>125</v>
+      </c>
+      <c r="C132" t="s">
+        <v>125</v>
+      </c>
+      <c r="D132" t="s">
         <v>292</v>
       </c>
-      <c r="G131"/>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
-        <v>174</v>
-      </c>
-      <c r="B132" t="s">
-        <v>125</v>
-      </c>
-      <c r="C132" t="s">
-        <v>125</v>
-      </c>
-      <c r="D132" t="s">
+      <c r="E132" t="s">
         <v>293</v>
       </c>
-      <c r="E132" t="s">
+      <c r="F132" t="s">
+        <v>291</v>
+      </c>
+      <c r="G132"/>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A133" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B133" t="s">
+        <v>125</v>
+      </c>
+      <c r="C133" t="s">
+        <v>125</v>
+      </c>
+      <c r="D133" t="s">
         <v>294</v>
       </c>
-      <c r="F132" t="s">
-        <v>292</v>
-      </c>
-      <c r="G132"/>
-    </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
-        <v>174</v>
-      </c>
-      <c r="B133" t="s">
-        <v>125</v>
-      </c>
-      <c r="C133" t="s">
-        <v>125</v>
-      </c>
-      <c r="D133" t="s">
+      <c r="E133" t="s">
         <v>295</v>
       </c>
-      <c r="E133" t="s">
+      <c r="F133" t="s">
+        <v>291</v>
+      </c>
+      <c r="G133"/>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A134" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B134" t="s">
+        <v>125</v>
+      </c>
+      <c r="C134" t="s">
+        <v>125</v>
+      </c>
+      <c r="D134" t="s">
         <v>296</v>
       </c>
-      <c r="F133" t="s">
-        <v>292</v>
-      </c>
-      <c r="G133"/>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>174</v>
-      </c>
-      <c r="B134" t="s">
-        <v>125</v>
-      </c>
-      <c r="C134" t="s">
-        <v>125</v>
-      </c>
-      <c r="D134" t="s">
+      <c r="E134" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="E134" s="6" t="s">
-        <v>298</v>
-      </c>
       <c r="F134" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G134"/>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
-        <v>174</v>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A135" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B135" t="s">
         <v>125</v>
@@ -4405,16 +4402,16 @@
         <v>152</v>
       </c>
       <c r="E135" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F135" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G135"/>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>174</v>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A136" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B136" t="s">
         <v>125</v>
@@ -4426,16 +4423,16 @@
         <v>153</v>
       </c>
       <c r="E136" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F136" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G136"/>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>174</v>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A137" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B137" t="s">
         <v>125</v>
@@ -4447,16 +4444,16 @@
         <v>154</v>
       </c>
       <c r="E137" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F137" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G137"/>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>174</v>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A138" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B138" t="s">
         <v>125</v>
@@ -4468,16 +4465,16 @@
         <v>155</v>
       </c>
       <c r="E138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F138" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G138"/>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>174</v>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A139" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B139" t="s">
         <v>125</v>
@@ -4489,16 +4486,16 @@
         <v>156</v>
       </c>
       <c r="E139" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F139" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G139"/>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>174</v>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A140" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B140" t="s">
         <v>125</v>
@@ -4510,16 +4507,16 @@
         <v>157</v>
       </c>
       <c r="E140" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F140" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G140"/>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>174</v>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A141" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B141" t="s">
         <v>125</v>
@@ -4531,16 +4528,16 @@
         <v>158</v>
       </c>
       <c r="E141" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F141" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G141"/>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
-        <v>174</v>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A142" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B142" t="s">
         <v>125</v>
@@ -4552,16 +4549,16 @@
         <v>159</v>
       </c>
       <c r="E142" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F142" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G142"/>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
-        <v>174</v>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A143" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B143" t="s">
         <v>125</v>
@@ -4573,16 +4570,16 @@
         <v>160</v>
       </c>
       <c r="E143" s="6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F143" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G143"/>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A144" t="s">
-        <v>174</v>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A144" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B144" t="s">
         <v>125</v>
@@ -4594,16 +4591,16 @@
         <v>161</v>
       </c>
       <c r="E144" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F144" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G144"/>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
-        <v>174</v>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A145" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B145" t="s">
         <v>125</v>
@@ -4615,58 +4612,58 @@
         <v>162</v>
       </c>
       <c r="E145" t="s">
+        <v>307</v>
+      </c>
+      <c r="F145" t="s">
+        <v>183</v>
+      </c>
+      <c r="G145"/>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A146" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B146" t="s">
+        <v>125</v>
+      </c>
+      <c r="C146" t="s">
+        <v>125</v>
+      </c>
+      <c r="D146" t="s">
         <v>308</v>
       </c>
-      <c r="F145" t="s">
-        <v>184</v>
-      </c>
-      <c r="G145"/>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A146" t="s">
-        <v>174</v>
-      </c>
-      <c r="B146" t="s">
-        <v>125</v>
-      </c>
-      <c r="C146" t="s">
-        <v>125</v>
-      </c>
-      <c r="D146" t="s">
+      <c r="E146" t="s">
         <v>309</v>
       </c>
-      <c r="E146" t="s">
+      <c r="F146" t="s">
+        <v>183</v>
+      </c>
+      <c r="G146"/>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A147" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B147" t="s">
+        <v>125</v>
+      </c>
+      <c r="C147" t="s">
+        <v>125</v>
+      </c>
+      <c r="D147" t="s">
         <v>310</v>
       </c>
-      <c r="F146" t="s">
-        <v>184</v>
-      </c>
-      <c r="G146"/>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A147" t="s">
-        <v>174</v>
-      </c>
-      <c r="B147" t="s">
-        <v>125</v>
-      </c>
-      <c r="C147" t="s">
-        <v>125</v>
-      </c>
-      <c r="D147" t="s">
+      <c r="E147" t="s">
         <v>311</v>
       </c>
-      <c r="E147" t="s">
-        <v>312</v>
-      </c>
       <c r="F147" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G147"/>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
-        <v>174</v>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A148" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B148" t="s">
         <v>125</v>
@@ -4678,58 +4675,58 @@
         <v>163</v>
       </c>
       <c r="E148" t="s">
+        <v>312</v>
+      </c>
+      <c r="F148" t="s">
+        <v>183</v>
+      </c>
+      <c r="G148"/>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A149" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B149" t="s">
+        <v>125</v>
+      </c>
+      <c r="C149" t="s">
+        <v>125</v>
+      </c>
+      <c r="D149" t="s">
         <v>313</v>
       </c>
-      <c r="F148" t="s">
-        <v>184</v>
-      </c>
-      <c r="G148"/>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
-        <v>174</v>
-      </c>
-      <c r="B149" t="s">
-        <v>125</v>
-      </c>
-      <c r="C149" t="s">
-        <v>125</v>
-      </c>
-      <c r="D149" t="s">
+      <c r="E149" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="E149" s="6" t="s">
+      <c r="F149" t="s">
+        <v>195</v>
+      </c>
+      <c r="G149"/>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A150" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B150" t="s">
+        <v>125</v>
+      </c>
+      <c r="C150" t="s">
+        <v>125</v>
+      </c>
+      <c r="D150" t="s">
         <v>315</v>
       </c>
-      <c r="F149" t="s">
-        <v>196</v>
-      </c>
-      <c r="G149"/>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
-        <v>174</v>
-      </c>
-      <c r="B150" t="s">
-        <v>125</v>
-      </c>
-      <c r="C150" t="s">
-        <v>125</v>
-      </c>
-      <c r="D150" t="s">
-        <v>316</v>
-      </c>
       <c r="E150" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F150" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G150"/>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
-        <v>174</v>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A151" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B151" t="s">
         <v>125</v>
@@ -4741,16 +4738,16 @@
         <v>165</v>
       </c>
       <c r="E151" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F151" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G151"/>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
-        <v>174</v>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A152" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B152" t="s">
         <v>125</v>
@@ -4762,10 +4759,10 @@
         <v>164</v>
       </c>
       <c r="E152" s="6" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F152" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G152"/>
     </row>

</xml_diff>